<commit_message>
updated results - NG reforming
</commit_message>
<xml_diff>
--- a/CCU/EtOH/analyses/parameter_distributions/10_full_samples.xlsx
+++ b/CCU/EtOH/analyses/parameter_distributions/10_full_samples.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL12"/>
+  <dimension ref="A1:BW12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,112 +629,167 @@
       </c>
       <c r="AQ1" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="AR1" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="AS1" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="AT1" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="AU1" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="AV1" t="inlineStr">
         <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>C3</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>C3</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>D2</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="BL1" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>B2</t>
         </is>
       </c>
     </row>
@@ -931,132 +986,187 @@
       </c>
       <c r="AM2" t="inlineStr">
         <is>
+          <t>Methanol unit price</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>Methanol GWP</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>CCU credit</t>
+        </is>
+      </c>
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>CCU credit years</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
           <t>Catalyst_MeOH unit price</t>
         </is>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AR2" t="inlineStr">
         <is>
           <t xml:space="preserve">Heat integration split recycled </t>
         </is>
       </c>
-      <c r="AO2" t="inlineStr">
+      <c r="AS2" t="inlineStr">
         <is>
           <t>MeOH conversion</t>
         </is>
       </c>
-      <c r="AP2" t="inlineStr">
+      <c r="AT2" t="inlineStr">
         <is>
           <t>MeOH conversion WHSV</t>
         </is>
       </c>
-      <c r="AQ2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t>MeOH conversion catalyst density</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t>MeOH conversion catalyst longevity</t>
         </is>
       </c>
-      <c r="AS2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>MeOH conversion porosity</t>
         </is>
       </c>
-      <c r="AT2" t="inlineStr">
-        <is>
-          <t>Methanol unit price</t>
-        </is>
-      </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>Methanol GWP</t>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>Electrolyzer stack longevity</t>
         </is>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="AY2" t="inlineStr">
         <is>
           <t>Electrolyzer stack F_BM</t>
         </is>
       </c>
-      <c r="AX2" t="inlineStr">
+      <c r="AZ2" t="inlineStr">
         <is>
           <t>Electrolyzer mechanical BOP F_BM</t>
         </is>
       </c>
-      <c r="AY2" t="inlineStr">
+      <c r="BA2" t="inlineStr">
         <is>
           <t>Electrolyzer electrical BOP F_BM</t>
         </is>
       </c>
-      <c r="AZ2" t="inlineStr">
+      <c r="BB2" t="inlineStr">
         <is>
           <t>Electrolyzer base_power_per_hydrogen_flow</t>
         </is>
       </c>
-      <c r="BA2" t="inlineStr">
+      <c r="BC2" t="inlineStr">
         <is>
           <t>Oxygen unit price</t>
         </is>
       </c>
-      <c r="BB2" t="inlineStr">
+      <c r="BD2" t="inlineStr">
         <is>
           <t>Oxygen GWP</t>
         </is>
       </c>
-      <c r="BC2" t="inlineStr">
+      <c r="BE2" t="inlineStr">
         <is>
           <t>Hydrogen unit price (conventional)</t>
         </is>
       </c>
-      <c r="BD2" t="inlineStr">
+      <c r="BF2" t="inlineStr">
         <is>
           <t>Hydrogen GWP (conventional)</t>
         </is>
       </c>
-      <c r="BE2" t="inlineStr">
+      <c r="BG2" t="inlineStr">
         <is>
           <t>Hydrogen unit price (renewable)</t>
         </is>
       </c>
-      <c r="BF2" t="inlineStr">
+      <c r="BH2" t="inlineStr">
         <is>
           <t>Hydrogen GWP (renewable)</t>
         </is>
       </c>
-      <c r="BG2" t="inlineStr">
+      <c r="BI2" t="inlineStr">
         <is>
           <t>Electricity unit price (conventional)</t>
         </is>
       </c>
-      <c r="BH2" t="inlineStr">
+      <c r="BJ2" t="inlineStr">
         <is>
           <t>Electricity GWP (conventional)</t>
         </is>
       </c>
-      <c r="BI2" t="inlineStr">
+      <c r="BK2" t="inlineStr">
         <is>
           <t>Electricity unit price (renewable)</t>
         </is>
       </c>
-      <c r="BJ2" t="inlineStr">
+      <c r="BL2" t="inlineStr">
         <is>
           <t>Electricity GWP (renewable)</t>
         </is>
       </c>
-      <c r="BK2" t="inlineStr">
-        <is>
-          <t>CCU credit</t>
-        </is>
-      </c>
-      <c r="BL2" t="inlineStr">
-        <is>
-          <t>CCU credit years</t>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>Bi-reforming GHSV</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>Bi-reforming catalyst price</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr">
+        <is>
+          <t>Bi-reforming catalyst longevity</t>
+        </is>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>Bi-reforming residence time</t>
+        </is>
+      </c>
+      <c r="BQ2" t="inlineStr">
+        <is>
+          <t>Bi-reforming conversion</t>
+        </is>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>Methane membrane separator longevity</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr">
+        <is>
+          <t>MeOH synthesis WHSV</t>
+        </is>
+      </c>
+      <c r="BT2" t="inlineStr">
+        <is>
+          <t>MeOH synthesis catalyst density</t>
+        </is>
+      </c>
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>MeOH synthesis catalyst longevity</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>MeOH synthesis porosity</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>MeOH synthesis catalyst price</t>
         </is>
       </c>
     </row>
@@ -1068,190 +1178,223 @@
         <v>84597.14844379794</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1925204102288536</v>
+        <v>0.1871583703755017</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3670407285669111</v>
+        <v>0.370871242423073</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2029702832911175</v>
+        <v>0.2076382788862444</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2093602221129102</v>
+        <v>0.2019072514227982</v>
       </c>
       <c r="G3" t="n">
-        <v>0.05081190345545245</v>
+        <v>0.03927911202641908</v>
       </c>
       <c r="H3" t="n">
-        <v>335.7241444450513</v>
+        <v>308.2795258652822</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1696469573274428</v>
+        <v>0.2736469573274428</v>
       </c>
       <c r="J3" t="n">
-        <v>0.08532625204247722</v>
+        <v>0.09332625204247721</v>
       </c>
       <c r="K3" t="n">
-        <v>0.09087186479789097</v>
+        <v>0.08400681490809124</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1734632907484533</v>
+        <v>0.1209151423656199</v>
       </c>
       <c r="M3" t="n">
-        <v>0.721335173957636</v>
+        <v>0.8614635696451921</v>
       </c>
       <c r="N3" t="n">
-        <v>0.4669493095069002</v>
+        <v>0.4179002270197629</v>
       </c>
       <c r="O3" t="n">
-        <v>0.0904863453240442</v>
+        <v>0.1182436670042651</v>
       </c>
       <c r="P3" t="n">
-        <v>1.088888711746503</v>
+        <v>0.9928140974265456</v>
       </c>
       <c r="Q3" t="n">
-        <v>1.051047168774263</v>
+        <v>0.7589006953408131</v>
       </c>
       <c r="R3" t="n">
-        <v>0.7501269540177451</v>
+        <v>1.007709208336811</v>
       </c>
       <c r="S3" t="n">
-        <v>2.342166496311937</v>
+        <v>2.256378299567765</v>
       </c>
       <c r="T3" t="n">
         <v>0.1244279737872541</v>
       </c>
       <c r="U3" t="n">
-        <v>3.423071997669246</v>
+        <v>3.656829885748675</v>
       </c>
       <c r="V3" t="n">
-        <v>0.001017402672440528</v>
+        <v>0.001178208501871612</v>
       </c>
       <c r="W3" t="n">
-        <v>0.002490126472890004</v>
+        <v>0.002299805683687567</v>
       </c>
       <c r="X3" t="n">
         <v>-0.05544325125771765</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.1979086880874392</v>
+        <v>0.228777747051153</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.01304325825705594</v>
+        <v>0.02445576162301251</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.1094788121033815</v>
+        <v>0.0944416622087253</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.8521782764619421</v>
+        <v>0.9104357624572863</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.9222424033748993</v>
+        <v>0.9393029834477197</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.8129632430445002</v>
+        <v>0.8711563814723392</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.861515743068468</v>
+        <v>0.8093781184622127</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.8049020644797195</v>
+        <v>0.7943415855806782</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.8724814277304811</v>
+        <v>0.8564814277304811</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.7754811245662412</v>
+        <v>0.9284811245662412</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.09235563061709191</v>
+        <v>0.09846103174087616</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.3084030353581323</v>
+        <v>0.3182838530901849</v>
       </c>
       <c r="AK3" t="n">
-        <v>0.3692069437447866</v>
+        <v>0.3371389570954509</v>
       </c>
       <c r="AL3" t="n">
-        <v>1.264841603120028</v>
+        <v>1.610441603120029</v>
       </c>
       <c r="AM3" t="n">
-        <v>35.05433310351172</v>
+        <v>0.3377099209825416</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.6542891562350482</v>
+        <v>0.6593441454553013</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.2143628647531628</v>
+        <v>108.6227021894156</v>
       </c>
       <c r="AP3" t="n">
-        <v>2.920393589708778</v>
+        <v>11.1845197741048</v>
       </c>
       <c r="AQ3" t="n">
-        <v>1907.02714688312</v>
+        <v>33.82094422382145</v>
       </c>
       <c r="AR3" t="n">
-        <v>8539.81206249356</v>
+        <v>0.5912085201695847</v>
       </c>
       <c r="AS3" t="n">
-        <v>0.4374592470145919</v>
+        <v>0.2130580384542483</v>
       </c>
       <c r="AT3" t="n">
-        <v>0.37367340144707</v>
+        <v>3.150703881146161</v>
       </c>
       <c r="AU3" t="n">
-        <v>0.571021505991228</v>
+        <v>1747.522712300741</v>
       </c>
       <c r="AV3" t="n">
-        <v>10.77160751421775</v>
+        <v>7902.049636799634</v>
       </c>
       <c r="AW3" t="n">
-        <v>0.8998592189795936</v>
+        <v>0.5560450568439125</v>
       </c>
       <c r="AX3" t="n">
-        <v>1.324614547622519</v>
+        <v>10.50190169246766</v>
       </c>
       <c r="AY3" t="n">
-        <v>1.130619216875462</v>
+        <v>0.8368669679728311</v>
       </c>
       <c r="AZ3" t="n">
-        <v>52.63641345952287</v>
+        <v>1.218506549435062</v>
       </c>
       <c r="BA3" t="n">
-        <v>0.2084966751010106</v>
+        <v>1.082254510548985</v>
       </c>
       <c r="BB3" t="n">
-        <v>0.1895325516912957</v>
+        <v>51.76229720101996</v>
       </c>
       <c r="BC3" t="n">
-        <v>0.9900350709420646</v>
+        <v>0.1849948654977555</v>
       </c>
       <c r="BD3" t="n">
-        <v>11.67015707015146</v>
+        <v>0.182286797312954</v>
       </c>
       <c r="BE3" t="n">
-        <v>3.566632930334531</v>
+        <v>0.9592028402592874</v>
       </c>
       <c r="BF3" t="n">
-        <v>0.8164133307214775</v>
+        <v>12.3527678782843</v>
       </c>
       <c r="BG3" t="n">
-        <v>0.1014725580948233</v>
+        <v>3.502405113365867</v>
       </c>
       <c r="BH3" t="n">
-        <v>0.3877712270613838</v>
+        <v>0.8045402722639531</v>
       </c>
       <c r="BI3" t="n">
-        <v>0.02745142226367713</v>
+        <v>0.0954356982457837</v>
       </c>
       <c r="BJ3" t="n">
-        <v>0.0190367903797256</v>
+        <v>0.3777333178972909</v>
       </c>
       <c r="BK3" t="n">
-        <v>87.52886114867225</v>
+        <v>0.03384813736219044</v>
       </c>
       <c r="BL3" t="n">
-        <v>13.33571675667693</v>
+        <v>0.01720435232565992</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>56.18893409231589</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>34.71485775303651</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>7553.60146247101</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>5.167634105605024e-05</v>
+      </c>
+      <c r="BQ3" t="n">
+        <v>0.7402309151609334</v>
+      </c>
+      <c r="BR3" t="n">
+        <v>7.157144623942377</v>
+      </c>
+      <c r="BS3" t="n">
+        <v>3.163853736237803</v>
+      </c>
+      <c r="BT3" t="n">
+        <v>2017.587345911872</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>7174.754611871308</v>
+      </c>
+      <c r="BV3" t="n">
+        <v>0.5149258200223585</v>
+      </c>
+      <c r="BW3" t="n">
+        <v>29.6611479959961</v>
       </c>
     </row>
     <row r="4">
@@ -1259,193 +1402,226 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>87803.04413608434</v>
+        <v>70897.61624334093</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1969403459193038</v>
+        <v>0.2104126573791735</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3748139406789477</v>
+        <v>0.3632852430969284</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2117767852026442</v>
+        <v>0.206092812456228</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1933842788367025</v>
+        <v>0.1980752101947252</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04969513901964473</v>
+        <v>0.05803329226712817</v>
       </c>
       <c r="H4" t="n">
-        <v>330.5251951163937</v>
+        <v>323.2256944192465</v>
       </c>
       <c r="I4" t="n">
-        <v>0.2067587789998857</v>
+        <v>0.2457587789998857</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1035825605074916</v>
+        <v>0.1075825605074916</v>
       </c>
       <c r="K4" t="n">
-        <v>0.08258397991608507</v>
+        <v>0.09392086088618615</v>
       </c>
       <c r="L4" t="n">
         <v>0.1369786441694977</v>
       </c>
       <c r="M4" t="n">
-        <v>0.9872077614323014</v>
+        <v>0.8821114646666345</v>
       </c>
       <c r="N4" t="n">
-        <v>0.4211891176957263</v>
+        <v>0.4538885060204845</v>
       </c>
       <c r="O4" t="n">
-        <v>0.1076666332516859</v>
+        <v>0.1037013015830829</v>
       </c>
       <c r="P4" t="n">
-        <v>1.396201737719076</v>
+        <v>1.25208981623914</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.9149398519074223</v>
+        <v>0.8053849243698785</v>
       </c>
       <c r="R4" t="n">
-        <v>0.8020430472100042</v>
+        <v>0.8756379770154515</v>
       </c>
       <c r="S4" t="n">
-        <v>1.729152901282399</v>
+        <v>1.900729294770741</v>
       </c>
       <c r="T4" t="n">
-        <v>0.1277678948416888</v>
+        <v>0.1400261586408792</v>
       </c>
       <c r="U4" t="n">
-        <v>3.829344661011703</v>
+        <v>3.72732440204119</v>
       </c>
       <c r="V4" t="n">
-        <v>0.001070320321164345</v>
+        <v>0.0008945967061012061</v>
       </c>
       <c r="W4" t="n">
-        <v>0.002415629368731918</v>
+        <v>0.00249337234393538</v>
       </c>
       <c r="X4" t="n">
-        <v>-0.05900966933004583</v>
+        <v>-0.06085966918257182</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.2360041264900248</v>
+        <v>0.2044930282779965</v>
       </c>
       <c r="Z4" t="n">
-        <v>0.01873172167680322</v>
+        <v>0.01602021290663006</v>
       </c>
       <c r="AA4" t="n">
-        <v>0.1029937267093041</v>
+        <v>0.1069853913315458</v>
       </c>
       <c r="AB4" t="n">
-        <v>0.8911779598445312</v>
+        <v>0.8682844721248908</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.9474510163236219</v>
+        <v>0.9510431959459896</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.8418497186092947</v>
+        <v>0.8158555651957647</v>
       </c>
       <c r="AE4" t="n">
-        <v>0.873692865856991</v>
+        <v>0.9196023948272567</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.815595719526939</v>
+        <v>0.798128426996225</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.8182658412554833</v>
+        <v>0.8022658412554833</v>
       </c>
       <c r="AH4" t="n">
-        <v>0.8714298290543484</v>
+        <v>0.8544298290543484</v>
       </c>
       <c r="AI4" t="n">
-        <v>0.1015496859680186</v>
+        <v>0.1046347103484591</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0.280545128566194</v>
+        <v>0.2514042159823929</v>
       </c>
       <c r="AK4" t="n">
-        <v>0.3304005894647825</v>
+        <v>0.3559686834528957</v>
       </c>
       <c r="AL4" t="n">
-        <v>1.547453351742964</v>
+        <v>1.432253351742964</v>
       </c>
       <c r="AM4" t="n">
-        <v>35.49687049157967</v>
+        <v>0.3727894200503311</v>
       </c>
       <c r="AN4" t="n">
-        <v>0.5068800083381032</v>
+        <v>0.5220204160177329</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.2296693203060922</v>
+        <v>77.98112460279741</v>
       </c>
       <c r="AP4" t="n">
-        <v>2.677089664630135</v>
+        <v>12.8538081074725</v>
       </c>
       <c r="AQ4" t="n">
-        <v>1757.960670408276</v>
+        <v>38.37420211656551</v>
       </c>
       <c r="AR4" t="n">
-        <v>7030.599125762525</v>
+        <v>0.492282323959648</v>
       </c>
       <c r="AS4" t="n">
-        <v>0.5647852798522613</v>
+        <v>0.2280928986018644</v>
       </c>
       <c r="AT4" t="n">
-        <v>0.3526440054527611</v>
+        <v>2.89091682938196</v>
       </c>
       <c r="AU4" t="n">
-        <v>0.6104480530226349</v>
+        <v>1921.808008870347</v>
       </c>
       <c r="AV4" t="n">
-        <v>8.671878603215722</v>
+        <v>6836.909090775275</v>
       </c>
       <c r="AW4" t="n">
-        <v>1.156202912811322</v>
+        <v>0.4961093513465166</v>
       </c>
       <c r="AX4" t="n">
-        <v>1.368189901062692</v>
+        <v>9.43701158699983</v>
       </c>
       <c r="AY4" t="n">
-        <v>1.050137651157751</v>
+        <v>0.8986326377149602</v>
       </c>
       <c r="AZ4" t="n">
-        <v>51.42871415490094</v>
+        <v>1.367759154600287</v>
       </c>
       <c r="BA4" t="n">
-        <v>0.221856831698473</v>
+        <v>1.058278323756217</v>
       </c>
       <c r="BB4" t="n">
-        <v>0.1462763734355863</v>
+        <v>52.18226506037517</v>
       </c>
       <c r="BC4" t="n">
-        <v>1.028994121432928</v>
+        <v>0.2431130778130659</v>
       </c>
       <c r="BD4" t="n">
-        <v>10.94055092240736</v>
+        <v>0.1963912047742897</v>
       </c>
       <c r="BE4" t="n">
-        <v>4.571383387055687</v>
+        <v>1.051019266454644</v>
       </c>
       <c r="BF4" t="n">
-        <v>0.3028243073546393</v>
+        <v>11.70618799806167</v>
       </c>
       <c r="BG4" t="n">
-        <v>0.0856859815192344</v>
+        <v>3.716383945200437</v>
       </c>
       <c r="BH4" t="n">
-        <v>0.4517346748757211</v>
+        <v>0.4053537909108068</v>
       </c>
       <c r="BI4" t="n">
-        <v>0.03576188777843114</v>
+        <v>0.08129686733961951</v>
       </c>
       <c r="BJ4" t="n">
-        <v>0.01581465559668515</v>
+        <v>0.4264939888933597</v>
       </c>
       <c r="BK4" t="n">
-        <v>95.28961411696966</v>
+        <v>0.03500222956149818</v>
       </c>
       <c r="BL4" t="n">
-        <v>12.18465945749028</v>
+        <v>0.01992789621133913</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>67.03219014539314</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>30.71153672047636</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>8388.172882093986</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>5.946275375075293e-05</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>0.764507588401756</v>
+      </c>
+      <c r="BR4" t="n">
+        <v>7.419385583653538</v>
+      </c>
+      <c r="BS4" t="n">
+        <v>2.86993028196951</v>
+      </c>
+      <c r="BT4" t="n">
+        <v>1976.430551127254</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>6808.242124117703</v>
+      </c>
+      <c r="BV4" t="n">
+        <v>0.505563875531078</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>32.97178412868111</v>
       </c>
     </row>
     <row r="5">
@@ -1456,190 +1632,223 @@
         <v>79103.23046012702</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2022826075524691</v>
+        <v>0.2067945532624381</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3453452481018596</v>
+        <v>0.3865835148883773</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2007635820929966</v>
+        <v>0.1975138409284723</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2006523018719264</v>
+        <v>0.1961057939075883</v>
       </c>
       <c r="G5" t="n">
-        <v>0.03964849398680058</v>
+        <v>0.04281832753457662</v>
       </c>
       <c r="H5" t="n">
-        <v>324.7086957803322</v>
+        <v>335.4894896784338</v>
       </c>
       <c r="I5" t="n">
-        <v>0.2577874888071545</v>
+        <v>0.2317874888071545</v>
       </c>
       <c r="J5" t="n">
-        <v>0.09218373153518364</v>
+        <v>0.08818373153518365</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1013018507337248</v>
+        <v>0.08926113519389989</v>
       </c>
       <c r="L5" t="n">
-        <v>0.1501786046486363</v>
+        <v>0.1560172878022845</v>
       </c>
       <c r="M5" t="n">
-        <v>0.7594894685690091</v>
+        <v>0.8295536664127872</v>
       </c>
       <c r="N5" t="n">
         <v>0.3660887541488831</v>
       </c>
       <c r="O5" t="n">
-        <v>0.08454748544920931</v>
+        <v>0.09644348045501827</v>
       </c>
       <c r="P5" t="n">
-        <v>1.181111111933329</v>
+        <v>1.373260340573244</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.8049385927861517</v>
+        <v>0.8779752111445142</v>
       </c>
       <c r="R5" t="n">
-        <v>0.9283086050000724</v>
+        <v>0.8179162102919013</v>
       </c>
       <c r="S5" t="n">
-        <v>2.104285849908569</v>
+        <v>2.361650440141081</v>
       </c>
       <c r="T5" t="n">
-        <v>0.1147819268364045</v>
+        <v>0.1300846100953662</v>
       </c>
       <c r="U5" t="n">
-        <v>3.033384643771289</v>
+        <v>3.513905511143649</v>
       </c>
       <c r="V5" t="n">
-        <v>0.001209964581417656</v>
+        <v>0.001113788681882037</v>
       </c>
       <c r="W5" t="n">
-        <v>0.002342008586507841</v>
+        <v>0.002064365388583986</v>
       </c>
       <c r="X5" t="n">
-        <v>-0.04781027194876195</v>
+        <v>-0.05870341084882683</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.2053603415646125</v>
+        <v>0.2097793696565051</v>
       </c>
       <c r="Z5" t="n">
-        <v>0.02159690841745241</v>
+        <v>0.01702766332825626</v>
       </c>
       <c r="AA5" t="n">
-        <v>0.101780780502933</v>
+        <v>0.1031039453931276</v>
       </c>
       <c r="AB5" t="n">
-        <v>0.8343002193791179</v>
+        <v>0.8143158377646393</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.9408587816193315</v>
+        <v>0.9643233825359186</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.860492580307634</v>
+        <v>0.849387891119699</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.8468600438684203</v>
+        <v>0.8852474328709876</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.7855876149476404</v>
+        <v>0.8229163949530628</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.7873592057814963</v>
+        <v>0.7393592057814964</v>
       </c>
       <c r="AH5" t="n">
-        <v>0.9159179200758812</v>
+        <v>0.8479179200758812</v>
       </c>
       <c r="AI5" t="n">
-        <v>0.1079511876231142</v>
+        <v>0.1187223145022966</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0.2685478418228268</v>
+        <v>0.2766919320186305</v>
       </c>
       <c r="AK5" t="n">
-        <v>0.371423774531511</v>
+        <v>0.3478657624522924</v>
       </c>
       <c r="AL5" t="n">
-        <v>1.372368028390332</v>
+        <v>1.487568028390332</v>
       </c>
       <c r="AM5" t="n">
-        <v>31.69780259957569</v>
+        <v>0.3549798171355777</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.6011986389088743</v>
+        <v>0.5811586842785785</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.1925518366474663</v>
+        <v>89.71637372035059</v>
       </c>
       <c r="AP5" t="n">
-        <v>2.740298511610158</v>
+        <v>10.81640914411815</v>
       </c>
       <c r="AQ5" t="n">
-        <v>1780.109753904536</v>
+        <v>35.27033247143038</v>
       </c>
       <c r="AR5" t="n">
-        <v>7491.199990571404</v>
+        <v>0.6616835298110042</v>
       </c>
       <c r="AS5" t="n">
-        <v>0.5236671978731483</v>
+        <v>0.214843179704841</v>
       </c>
       <c r="AT5" t="n">
-        <v>0.3353312209071484</v>
+        <v>2.810698771345002</v>
       </c>
       <c r="AU5" t="n">
-        <v>0.6521618086875587</v>
+        <v>1824.036111968586</v>
       </c>
       <c r="AV5" t="n">
-        <v>9.795717645964837</v>
+        <v>8245.692164789196</v>
       </c>
       <c r="AW5" t="n">
-        <v>1.031522017866047</v>
+        <v>0.4775717425917127</v>
       </c>
       <c r="AX5" t="n">
-        <v>1.502760252552303</v>
+        <v>10.31682997233159</v>
       </c>
       <c r="AY5" t="n">
-        <v>0.9666862151926956</v>
+        <v>1.113854585195218</v>
       </c>
       <c r="AZ5" t="n">
-        <v>51.06092224392825</v>
+        <v>1.563319507510424</v>
       </c>
       <c r="BA5" t="n">
-        <v>0.2509994564419323</v>
+        <v>1.016277274286244</v>
       </c>
       <c r="BB5" t="n">
-        <v>0.1676148989629849</v>
+        <v>50.37028398078741</v>
       </c>
       <c r="BC5" t="n">
-        <v>1.016566508280964</v>
+        <v>0.2357044211319618</v>
       </c>
       <c r="BD5" t="n">
-        <v>11.0576423414548</v>
+        <v>0.1854768736112787</v>
       </c>
       <c r="BE5" t="n">
-        <v>4.106575085521752</v>
+        <v>1.030414236603048</v>
       </c>
       <c r="BF5" t="n">
-        <v>0.5562972997006265</v>
+        <v>9.903457003367981</v>
       </c>
       <c r="BG5" t="n">
-        <v>0.09302095975233456</v>
+        <v>4.634296038123745</v>
       </c>
       <c r="BH5" t="n">
-        <v>0.3728733184241269</v>
+        <v>0.5696680430981793</v>
       </c>
       <c r="BI5" t="n">
-        <v>0.02984571451275642</v>
+        <v>0.0932051230217639</v>
       </c>
       <c r="BJ5" t="n">
-        <v>0.02063398652778729</v>
+        <v>0.4445463003856545</v>
       </c>
       <c r="BK5" t="n">
-        <v>88.86309889693604</v>
+        <v>0.01698333650568816</v>
       </c>
       <c r="BL5" t="n">
-        <v>11.90129337467608</v>
+        <v>0.02101891676035229</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>57.84898869564302</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>32.1950405519213</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>6884.664450248869</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>4.961427059113953e-05</v>
+      </c>
+      <c r="BQ5" t="n">
+        <v>0.7553194183805353</v>
+      </c>
+      <c r="BR5" t="n">
+        <v>5.152429962811944</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>2.600584622784814</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>1908.181483461632</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>7598.752131793433</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>0.4667522536145086</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>30.46673224347605</v>
       </c>
     </row>
     <row r="6">
@@ -1647,22 +1856,22 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>81787.7005614308</v>
+        <v>87341.27878329399</v>
       </c>
       <c r="C6" t="n">
-        <v>0.2094586598458812</v>
+        <v>0.1961555879718531</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3567201470035738</v>
+        <v>0.3525547632777354</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2086000458092738</v>
+        <v>0.202595505070659</v>
       </c>
       <c r="F6" t="n">
         <v>0.2052164295910241</v>
       </c>
       <c r="G6" t="n">
-        <v>0.03623776688944703</v>
+        <v>0.05288304278629061</v>
       </c>
       <c r="H6" t="n">
         <v>342.053369907208</v>
@@ -1674,13 +1883,13 @@
         <v>0.1099292083761779</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1006660561174342</v>
+        <v>0.0804710736261153</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1518283862079623</v>
+        <v>0.1284736535933697</v>
       </c>
       <c r="M6" t="n">
-        <v>0.8957599209651532</v>
+        <v>0.7205994263557082</v>
       </c>
       <c r="N6" t="n">
         <v>0.3942883359341418</v>
@@ -1689,151 +1898,184 @@
         <v>0.1125263582701264</v>
       </c>
       <c r="P6" t="n">
-        <v>1.357271996911769</v>
+        <v>1.117085461111875</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.8793392447725987</v>
+        <v>1.025412481489324</v>
       </c>
       <c r="R6" t="n">
-        <v>0.965122345354874</v>
+        <v>0.7443375559385317</v>
       </c>
       <c r="S6" t="n">
         <v>2.42241072749828</v>
       </c>
       <c r="T6" t="n">
-        <v>0.1488310496659345</v>
+        <v>0.1345457113661073</v>
       </c>
       <c r="U6" t="n">
-        <v>3.366322430601092</v>
+        <v>4.078687458492343</v>
       </c>
       <c r="V6" t="n">
-        <v>0.001096084808003746</v>
+        <v>0.001221869266017548</v>
       </c>
       <c r="W6" t="n">
-        <v>0.002249209952934633</v>
+        <v>0.002199370196276145</v>
       </c>
       <c r="X6" t="n">
-        <v>-0.05774343321101012</v>
+        <v>-0.05109365843600489</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.2267595433988193</v>
+        <v>0.2008561415532789</v>
       </c>
       <c r="Z6" t="n">
-        <v>0.02273331026513571</v>
+        <v>0.01268239078010979</v>
       </c>
       <c r="AA6" t="n">
-        <v>0.09684462847451998</v>
+        <v>0.1014471606442194</v>
       </c>
       <c r="AB6" t="n">
-        <v>0.9019201562515629</v>
+        <v>0.7976919804618536</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.9181685712566765</v>
+        <v>0.945608080221699</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.8318800291222926</v>
+        <v>0.8780076435286763</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.7908688486417349</v>
+        <v>0.8372368201466619</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.7974820511084009</v>
+        <v>0.8343330021210441</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.8497601269939683</v>
+        <v>0.7697601269939682</v>
       </c>
       <c r="AH6" t="n">
-        <v>0.822540680647087</v>
+        <v>0.8735406806470869</v>
       </c>
       <c r="AI6" t="n">
-        <v>0.1191888842079433</v>
+        <v>0.0941946985619567</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0.2410978260651536</v>
+        <v>0.259100105764179</v>
       </c>
       <c r="AK6" t="n">
-        <v>0.3898367736965631</v>
+        <v>0.3254345394969753</v>
       </c>
       <c r="AL6" t="n">
-        <v>1.410103414151158</v>
+        <v>1.525303414151158</v>
       </c>
       <c r="AM6" t="n">
-        <v>38.5805947808016</v>
+        <v>0.347129191317988</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.6978368132668022</v>
+        <v>0.5780043617214833</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.2042333135683683</v>
+        <v>69.49499010368389</v>
       </c>
       <c r="AP6" t="n">
-        <v>3.175526025697674</v>
+        <v>11.91209682216081</v>
       </c>
       <c r="AQ6" t="n">
-        <v>1703.945334520654</v>
+        <v>32.74406586918334</v>
       </c>
       <c r="AR6" t="n">
-        <v>6950.783021047286</v>
+        <v>0.5850663347398638</v>
       </c>
       <c r="AS6" t="n">
-        <v>0.5152196334190726</v>
+        <v>0.2026653697173417</v>
       </c>
       <c r="AT6" t="n">
-        <v>0.3290039135592568</v>
+        <v>2.949016487857711</v>
       </c>
       <c r="AU6" t="n">
-        <v>0.5906514427077154</v>
+        <v>1637.454275823657</v>
       </c>
       <c r="AV6" t="n">
-        <v>11.87738327185806</v>
+        <v>7524.752321773119</v>
       </c>
       <c r="AW6" t="n">
-        <v>0.9416265607755323</v>
+        <v>0.5018982962241587</v>
       </c>
       <c r="AX6" t="n">
-        <v>1.581524420806664</v>
+        <v>9.925810877911568</v>
       </c>
       <c r="AY6" t="n">
-        <v>1.022646765997683</v>
+        <v>0.9836887939596766</v>
       </c>
       <c r="AZ6" t="n">
-        <v>51.70858307307807</v>
+        <v>1.425481856428382</v>
       </c>
       <c r="BA6" t="n">
-        <v>0.1886669582719591</v>
+        <v>0.8613056790676393</v>
       </c>
       <c r="BB6" t="n">
-        <v>0.1580154962798952</v>
+        <v>49.87667134870621</v>
       </c>
       <c r="BC6" t="n">
-        <v>0.973807368804924</v>
+        <v>0.2561203203926111</v>
       </c>
       <c r="BD6" t="n">
-        <v>11.38817735736677</v>
+        <v>0.1666008597732828</v>
       </c>
       <c r="BE6" t="n">
-        <v>3.881044864024374</v>
+        <v>1.077678578585079</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.4944390387528878</v>
+        <v>10.83500688929281</v>
       </c>
       <c r="BG6" t="n">
-        <v>0.08042846954224458</v>
+        <v>4.878634872544277</v>
       </c>
       <c r="BH6" t="n">
-        <v>0.4240060124466934</v>
+        <v>0.7823918396443323</v>
       </c>
       <c r="BI6" t="n">
-        <v>0.02444235091013108</v>
+        <v>0.08283861045018506</v>
       </c>
       <c r="BJ6" t="n">
-        <v>0.01869888954168182</v>
+        <v>0.4640312641902994</v>
       </c>
       <c r="BK6" t="n">
-        <v>80.81135015722626</v>
+        <v>0.01319759127086405</v>
       </c>
       <c r="BL6" t="n">
-        <v>12.29308385724452</v>
+        <v>0.01785751781389286</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>62.50392775290943</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>28.04628806148781</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>7268.918752049312</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>5.718831840622171e-05</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>0.7171752340099024</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>8.222402215997596</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>2.997463712957543</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>2090.151616792098</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>8109.590694266699</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>0.553432056553573</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>28.68050354723843</v>
       </c>
     </row>
     <row r="7">
@@ -1841,193 +2083,226 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>91927.32837790748</v>
+        <v>96899.6013865017</v>
       </c>
       <c r="C7" t="n">
-        <v>0.1731998515875273</v>
+        <v>0.2279267271186619</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3773436737302281</v>
+        <v>0.372520776798276</v>
       </c>
       <c r="E7" t="n">
-        <v>0.207047479071872</v>
+        <v>0.2021882606206093</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2029642523305303</v>
+        <v>0.2003867074176024</v>
       </c>
       <c r="G7" t="n">
-        <v>0.04443218895052526</v>
+        <v>0.04114430985568943</v>
       </c>
       <c r="H7" t="n">
-        <v>353.2421778387961</v>
+        <v>328.5243541832393</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1970516606175751</v>
+        <v>0.1710516606175751</v>
       </c>
       <c r="J7" t="n">
         <v>0.1150956415677746</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0890391422247139</v>
+        <v>0.1008672568297575</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1242128910377649</v>
+        <v>0.1709223562669502</v>
       </c>
       <c r="M7" t="n">
-        <v>0.8658899036275578</v>
+        <v>1.006018299315114</v>
       </c>
       <c r="N7" t="n">
-        <v>0.4554362484640794</v>
+        <v>0.3573380834898047</v>
       </c>
       <c r="O7" t="n">
-        <v>0.103817643587654</v>
+        <v>0.09192164858184503</v>
       </c>
       <c r="P7" t="n">
-        <v>0.9786718490844626</v>
+        <v>1.314932999204314</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.7977414853596057</v>
+        <v>1.016851340434693</v>
       </c>
       <c r="R7" t="n">
-        <v>0.8445012539393206</v>
+        <v>1.102083508258387</v>
       </c>
       <c r="S7" t="n">
-        <v>1.928263806306044</v>
+        <v>2.014052003050214</v>
       </c>
       <c r="T7" t="n">
-        <v>0.1370356582834827</v>
+        <v>0.1278878260875293</v>
       </c>
       <c r="U7" t="n">
-        <v>3.198528276124672</v>
+        <v>3.847429489595184</v>
       </c>
       <c r="V7" t="n">
         <v>0.00116975003936704</v>
       </c>
       <c r="W7" t="n">
-        <v>0.002091300166484687</v>
+        <v>0.002004050221592327</v>
       </c>
       <c r="X7" t="n">
-        <v>-0.06437093491514642</v>
+        <v>-0.05642046398259117</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.201406051059478</v>
+        <v>0.1864810305801774</v>
       </c>
       <c r="Z7" t="n">
-        <v>0.01999285586081566</v>
+        <v>0.01893628380564527</v>
       </c>
       <c r="AA7" t="n">
-        <v>0.09518724030645281</v>
+        <v>0.09684890224757871</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.9104041448137278</v>
+        <v>0.8521419305551846</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.9561953119091675</v>
+        <v>0.9303904008987554</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.8912458818666862</v>
+        <v>0.867187889670245</v>
       </c>
       <c r="AE7" t="n">
-        <v>0.9147083127897548</v>
+        <v>0.8816299685991853</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.7766545307472331</v>
+        <v>0.802150903972543</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.7760462070902724</v>
+        <v>0.7280462070902725</v>
       </c>
       <c r="AH7" t="n">
-        <v>0.8992297299411925</v>
+        <v>0.8312297299411925</v>
       </c>
       <c r="AI7" t="n">
-        <v>0.1170253256150362</v>
+        <v>0.1041208634211041</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0.3260371974534487</v>
+        <v>0.2709908378224545</v>
       </c>
       <c r="AK7" t="n">
-        <v>0.3431532084144207</v>
+        <v>0.3867329917834308</v>
       </c>
       <c r="AL7" t="n">
-        <v>1.276216103783271</v>
+        <v>1.161016103783271</v>
       </c>
       <c r="AM7" t="n">
-        <v>37.40672429261388</v>
+        <v>0.3903190570551104</v>
       </c>
       <c r="AN7" t="n">
-        <v>0.6272849417031604</v>
+        <v>0.5540812905015148</v>
       </c>
       <c r="AO7" t="n">
-        <v>0.1800621711111643</v>
+        <v>83.48511110393116</v>
       </c>
       <c r="AP7" t="n">
-        <v>2.860800080649751</v>
+        <v>14.05282133238894</v>
       </c>
       <c r="AQ7" t="n">
-        <v>1560.941303704969</v>
+        <v>32.21045090343457</v>
       </c>
       <c r="AR7" t="n">
-        <v>7624.12249760717</v>
+        <v>0.6060023330370528</v>
       </c>
       <c r="AS7" t="n">
-        <v>0.4723941987857241</v>
+        <v>0.2404284094068565</v>
       </c>
       <c r="AT7" t="n">
-        <v>0.345997014974413</v>
+        <v>2.723282212835358</v>
       </c>
       <c r="AU7" t="n">
-        <v>0.5528954941372662</v>
+        <v>1809.963554445016</v>
       </c>
       <c r="AV7" t="n">
-        <v>10.72382388395935</v>
+        <v>7711.210584857156</v>
       </c>
       <c r="AW7" t="n">
-        <v>1.016651350425377</v>
+        <v>0.5421010134753503</v>
       </c>
       <c r="AX7" t="n">
-        <v>1.385199165420872</v>
+        <v>10.03767511174545</v>
       </c>
       <c r="AY7" t="n">
-        <v>0.9303510153716965</v>
+        <v>1.081887689988818</v>
       </c>
       <c r="AZ7" t="n">
-        <v>50.8290752374222</v>
+        <v>1.269121595021061</v>
       </c>
       <c r="BA7" t="n">
-        <v>0.2192056282747384</v>
+        <v>1.048497844621124</v>
       </c>
       <c r="BB7" t="n">
-        <v>0.160257359578072</v>
+        <v>50.54372755570868</v>
       </c>
       <c r="BC7" t="n">
-        <v>1.057053773791037</v>
+        <v>0.2186067688116077</v>
       </c>
       <c r="BD7" t="n">
-        <v>9.534462730393503</v>
+        <v>0.1782126089565191</v>
       </c>
       <c r="BE7" t="n">
-        <v>4.806223224364214</v>
+        <v>1.042300821798483</v>
       </c>
       <c r="BF7" t="n">
-        <v>0.4473588615496776</v>
+        <v>10.64504357631001</v>
       </c>
       <c r="BG7" t="n">
-        <v>0.08831195179848902</v>
+        <v>3.775035480044923</v>
       </c>
       <c r="BH7" t="n">
-        <v>0.5079669507475991</v>
+        <v>0.4818659040150352</v>
       </c>
       <c r="BI7" t="n">
-        <v>0.02240518962656505</v>
+        <v>0.08498140736439913</v>
       </c>
       <c r="BJ7" t="n">
-        <v>0.01921076383358331</v>
+        <v>0.4157035713869789</v>
       </c>
       <c r="BK7" t="n">
-        <v>99.81155548531865</v>
+        <v>0.02226569678161323</v>
       </c>
       <c r="BL7" t="n">
-        <v>11.567912674001</v>
+        <v>0.0185536013533438</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>64.14959648436626</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>27.58034096155244</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>8590.624871290885</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>5.36659867284756e-05</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>0.7851422800301485</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>6.865710381226457</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>2.518385421560209</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>1809.972459457281</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>7468.086378252317</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>0.483090598073298</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>25.54296155141565</v>
       </c>
     </row>
     <row r="8">
@@ -2035,193 +2310,226 @@
         <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>73650.89638841698</v>
+        <v>81344.75003858029</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1853557056012885</v>
+        <v>0.1779697469803894</v>
       </c>
       <c r="D8" t="n">
-        <v>0.3857230130044803</v>
+        <v>0.3786808020433518</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2054572726861943</v>
+        <v>0.2105452247632791</v>
       </c>
       <c r="F8" t="n">
-        <v>0.2041046687838956</v>
+        <v>0.1949649376511811</v>
       </c>
       <c r="G8" t="n">
         <v>0.0457499648114454</v>
       </c>
       <c r="H8" t="n">
-        <v>309.1985671238709</v>
+        <v>316.1469329104059</v>
       </c>
       <c r="I8" t="n">
-        <v>0.216876204324823</v>
+        <v>0.2558762043248229</v>
       </c>
       <c r="J8" t="n">
-        <v>0.09925004513040256</v>
+        <v>0.1032500451304026</v>
       </c>
       <c r="K8" t="n">
-        <v>0.07768144292233992</v>
+        <v>0.08539225202537704</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1319454498646563</v>
+        <v>0.1261067667110081</v>
       </c>
       <c r="M8" t="n">
         <v>0.9594241699048637</v>
       </c>
       <c r="N8" t="n">
-        <v>0.4400810596658179</v>
+        <v>0.4891301421529552</v>
       </c>
       <c r="O8" t="n">
         <v>0.08220469409110871</v>
       </c>
       <c r="P8" t="n">
-        <v>1.139649784548963</v>
+        <v>1.091612477388985</v>
       </c>
       <c r="Q8" t="n">
-        <v>1.062891971106793</v>
+        <v>0.770745497673343</v>
       </c>
       <c r="R8" t="n">
-        <v>0.9157509942630212</v>
+        <v>0.9525484591657449</v>
       </c>
       <c r="S8" t="n">
-        <v>1.995308510017715</v>
+        <v>1.823732116529374</v>
       </c>
       <c r="T8" t="n">
-        <v>0.1387790367372862</v>
+        <v>0.1421444876781176</v>
       </c>
       <c r="U8" t="n">
-        <v>3.549286035822061</v>
+        <v>3.623197111270787</v>
       </c>
       <c r="V8" t="n">
-        <v>0.001130389387685748</v>
+        <v>0.001031121606268753</v>
       </c>
       <c r="W8" t="n">
-        <v>0.00227168468852242</v>
+        <v>0.002224477895711362</v>
       </c>
       <c r="X8" t="n">
-        <v>-0.05647156049372674</v>
+        <v>-0.04894912639943712</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.2148722224864882</v>
+        <v>0.2206919677726603</v>
       </c>
       <c r="Z8" t="n">
-        <v>0.01583186247175688</v>
+        <v>0.02755267899316134</v>
       </c>
       <c r="AA8" t="n">
         <v>0.1045766715557648</v>
       </c>
       <c r="AB8" t="n">
-        <v>0.872371238274633</v>
+        <v>0.8946192240224895</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.9315004420217139</v>
+        <v>0.9489109174680189</v>
       </c>
       <c r="AD8" t="n">
-        <v>0.8271738772289254</v>
+        <v>0.8351911864484947</v>
       </c>
       <c r="AE8" t="n">
-        <v>0.9018624399698658</v>
+        <v>0.7975172848309487</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.844123743211513</v>
+        <v>0.7810720067931854</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.7218921029549079</v>
+        <v>0.8338921029549079</v>
       </c>
       <c r="AH8" t="n">
-        <v>0.8006264233201109</v>
+        <v>0.885626423320111</v>
       </c>
       <c r="AI8" t="n">
-        <v>0.1002907549681459</v>
+        <v>0.1135326987462719</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0.2924326117180784</v>
+        <v>0.2864926949563153</v>
       </c>
       <c r="AK8" t="n">
-        <v>0.3278336781347531</v>
+        <v>0.3701465429791596</v>
       </c>
       <c r="AL8" t="n">
-        <v>1.557017750767649</v>
+        <v>1.269017750767649</v>
       </c>
       <c r="AM8" t="n">
-        <v>32.70703618998666</v>
+        <v>0.3389395387983116</v>
       </c>
       <c r="AN8" t="n">
-        <v>0.5703879745907561</v>
+        <v>0.6400500043140773</v>
       </c>
       <c r="AO8" t="n">
-        <v>0.2065068736124112</v>
+        <v>72.26218381851632</v>
       </c>
       <c r="AP8" t="n">
-        <v>3.411067834782437</v>
+        <v>11.71389936416684</v>
       </c>
       <c r="AQ8" t="n">
-        <v>1879.873079722041</v>
+        <v>27.96092020216054</v>
       </c>
       <c r="AR8" t="n">
-        <v>8773.139319466225</v>
+        <v>0.667666614875664</v>
       </c>
       <c r="AS8" t="n">
-        <v>0.5380986460668329</v>
+        <v>0.2199262479284209</v>
       </c>
       <c r="AT8" t="n">
-        <v>0.3685424368216583</v>
+        <v>2.54175062796872</v>
       </c>
       <c r="AU8" t="n">
-        <v>0.6048284323210731</v>
+        <v>1900.554644157477</v>
       </c>
       <c r="AV8" t="n">
-        <v>9.380354699674367</v>
+        <v>7136.100190491572</v>
       </c>
       <c r="AW8" t="n">
-        <v>0.8527519062420418</v>
+        <v>0.4221544090307138</v>
       </c>
       <c r="AX8" t="n">
-        <v>1.25907535740879</v>
+        <v>9.123734473976738</v>
       </c>
       <c r="AY8" t="n">
-        <v>1.113607169170197</v>
+        <v>1.001122927442642</v>
       </c>
       <c r="AZ8" t="n">
-        <v>51.96087711594453</v>
+        <v>1.458059294074784</v>
       </c>
       <c r="BA8" t="n">
-        <v>0.2358951755252846</v>
+        <v>1.175970610829405</v>
       </c>
       <c r="BB8" t="n">
-        <v>0.1715643754180617</v>
+        <v>52.56180401718786</v>
       </c>
       <c r="BC8" t="n">
-        <v>1.034584075830855</v>
+        <v>0.2255355884743643</v>
       </c>
       <c r="BD8" t="n">
-        <v>10.49342932960015</v>
+        <v>0.1587845335388926</v>
       </c>
       <c r="BE8" t="n">
-        <v>3.703942708711014</v>
+        <v>1.020443682651049</v>
       </c>
       <c r="BF8" t="n">
-        <v>0.7199700686851132</v>
+        <v>11.05876476791415</v>
       </c>
       <c r="BG8" t="n">
-        <v>0.08392610392103383</v>
+        <v>4.45098918015379</v>
       </c>
       <c r="BH8" t="n">
-        <v>0.4103725529740073</v>
+        <v>0.6295901569121325</v>
       </c>
       <c r="BI8" t="n">
-        <v>0.012041423862221</v>
+        <v>0.08845590721519703</v>
       </c>
       <c r="BJ8" t="n">
-        <v>0.02133158944551634</v>
+        <v>0.4832938233749795</v>
       </c>
       <c r="BK8" t="n">
-        <v>92.91787213426994</v>
+        <v>0.02815209944727037</v>
       </c>
       <c r="BL8" t="n">
-        <v>10.9915032601879</v>
+        <v>0.01959814252181651</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>53.99691135102356</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>32.31363865528282</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>9024.670213506797</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>6.138512616564498e-05</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>0.7684572896424475</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>8.022304646797091</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>3.071291906061973</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>2350.546430619906</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>7824.95625008085</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>0.4272439049329994</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>28.40162749260962</v>
       </c>
     </row>
     <row r="9">
@@ -2232,190 +2540,223 @@
         <v>75814.94095233959</v>
       </c>
       <c r="C9" t="n">
-        <v>0.224388263356919</v>
+        <v>0.2162570785072073</v>
       </c>
       <c r="D9" t="n">
-        <v>0.3535068242090964</v>
+        <v>0.3481285038033879</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2004598019602352</v>
+        <v>0.2098454158686839</v>
       </c>
       <c r="F9" t="n">
-        <v>0.2072364299540407</v>
+        <v>0.2009014908974344</v>
       </c>
       <c r="G9" t="n">
         <v>0.03781729420937079</v>
       </c>
       <c r="H9" t="n">
-        <v>320.9403903265902</v>
+        <v>332.154291854287</v>
       </c>
       <c r="I9" t="n">
-        <v>0.278201793551663</v>
+        <v>0.200201793551663</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1185805396367315</v>
+        <v>0.08658053963673147</v>
       </c>
       <c r="K9" t="n">
-        <v>0.09654310813013231</v>
+        <v>0.1037401421500932</v>
       </c>
       <c r="L9" t="n">
-        <v>0.1628789729267532</v>
+        <v>0.1512016066194569</v>
       </c>
       <c r="M9" t="n">
-        <v>1.031627115431883</v>
+        <v>0.7864024229786598</v>
       </c>
       <c r="N9" t="n">
-        <v>0.3819059451326954</v>
+        <v>0.4309550276198327</v>
       </c>
       <c r="O9" t="n">
-        <v>0.09459569982318233</v>
+        <v>0.1104570264975943</v>
       </c>
       <c r="P9" t="n">
-        <v>1.01353063427407</v>
+        <v>1.157642555754007</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.8566784843135921</v>
+        <v>1.07578833938868</v>
       </c>
       <c r="R9" t="n">
-        <v>1.012343636466983</v>
+        <v>0.9755461715642596</v>
       </c>
       <c r="S9" t="n">
-        <v>2.18923724015018</v>
+        <v>2.532390027126863</v>
       </c>
       <c r="T9" t="n">
-        <v>0.1448173331888827</v>
+        <v>0.1591946979315235</v>
       </c>
       <c r="U9" t="n">
-        <v>3.700166758381275</v>
+        <v>3.377783439632748</v>
       </c>
       <c r="V9" t="n">
-        <v>0.0009746231385139168</v>
+        <v>0.001116926776541004</v>
       </c>
       <c r="W9" t="n">
-        <v>0.002577498157617465</v>
+        <v>0.002399165307269959</v>
       </c>
       <c r="X9" t="n">
-        <v>-0.05403543038084218</v>
+        <v>-0.06422244212687128</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.1929377395844554</v>
+        <v>0.2149076219500513</v>
       </c>
       <c r="Z9" t="n">
-        <v>0.02084220130922362</v>
+        <v>0.02337691334340357</v>
       </c>
       <c r="AA9" t="n">
-        <v>0.0986425412994385</v>
+        <v>0.09589012055161014</v>
       </c>
       <c r="AB9" t="n">
-        <v>0.8091014847381015</v>
+        <v>0.9200170651903589</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.9603241143124913</v>
+        <v>0.9215857149616515</v>
       </c>
       <c r="AD9" t="n">
-        <v>0.8522594760712207</v>
+        <v>0.8414830371960113</v>
       </c>
       <c r="AE9" t="n">
-        <v>0.8437090131903674</v>
+        <v>0.8584037783156678</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.8102360622959464</v>
+        <v>0.8171188391060799</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.8353010704978102</v>
+        <v>0.8193010704978103</v>
       </c>
       <c r="AH9" t="n">
-        <v>0.8489952209424517</v>
+        <v>0.7809952209424517</v>
       </c>
       <c r="AI9" t="n">
-        <v>0.1233437115114708</v>
+        <v>0.1079372292132227</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0.2960658195157566</v>
+        <v>0.3030931921219228</v>
       </c>
       <c r="AK9" t="n">
-        <v>0.4000488166207219</v>
+        <v>0.374136101970784</v>
       </c>
       <c r="AL9" t="n">
-        <v>1.720640153880537</v>
+        <v>1.375040153880537</v>
       </c>
       <c r="AM9" t="n">
-        <v>29.11940606987772</v>
+        <v>0.3602522086572176</v>
       </c>
       <c r="AN9" t="n">
-        <v>0.6134467656392468</v>
+        <v>0.4764699343287807</v>
       </c>
       <c r="AO9" t="n">
-        <v>0.2211777809258922</v>
+        <v>91.65344102731682</v>
       </c>
       <c r="AP9" t="n">
-        <v>2.491835644062308</v>
+        <v>13.04583461570705</v>
       </c>
       <c r="AQ9" t="n">
-        <v>1833.375814511889</v>
+        <v>29.24914185625415</v>
       </c>
       <c r="AR9" t="n">
-        <v>8442.648383625878</v>
+        <v>0.642515097688423</v>
       </c>
       <c r="AS9" t="n">
-        <v>0.459588569069811</v>
+        <v>0.1845396701978044</v>
       </c>
       <c r="AT9" t="n">
-        <v>0.3809350347518861</v>
+        <v>2.96910127461892</v>
       </c>
       <c r="AU9" t="n">
-        <v>0.5282882503514874</v>
+        <v>1672.810770962639</v>
       </c>
       <c r="AV9" t="n">
-        <v>9.703144874344556</v>
+        <v>7823.861631720784</v>
       </c>
       <c r="AW9" t="n">
-        <v>0.968060054890107</v>
+        <v>0.4654110489581637</v>
       </c>
       <c r="AX9" t="n">
-        <v>1.464548814915299</v>
+        <v>8.689436441670075</v>
       </c>
       <c r="AY9" t="n">
-        <v>1.09571998528315</v>
+        <v>1.053978271558078</v>
       </c>
       <c r="AZ9" t="n">
-        <v>48.89614218749466</v>
+        <v>1.330933163885814</v>
       </c>
       <c r="BA9" t="n">
-        <v>0.2296776887239718</v>
+        <v>1.124885856558002</v>
       </c>
       <c r="BB9" t="n">
-        <v>0.1826922029885509</v>
+        <v>49.02372166958807</v>
       </c>
       <c r="BC9" t="n">
-        <v>1.048955244274581</v>
+        <v>0.2341491283737916</v>
       </c>
       <c r="BD9" t="n">
-        <v>10.77245558043574</v>
+        <v>0.1719834968865403</v>
       </c>
       <c r="BE9" t="n">
-        <v>4.201006143385981</v>
+        <v>0.9765257950248953</v>
       </c>
       <c r="BF9" t="n">
-        <v>0.07372964423525118</v>
+        <v>11.89429903564799</v>
       </c>
       <c r="BG9" t="n">
-        <v>0.09702372204241218</v>
+        <v>4.001431615411165</v>
       </c>
       <c r="BH9" t="n">
-        <v>0.4667515732790363</v>
+        <v>0.7160017521885274</v>
       </c>
       <c r="BI9" t="n">
-        <v>0.0177637702556217</v>
+        <v>0.08741826966621632</v>
       </c>
       <c r="BJ9" t="n">
-        <v>0.02029977639378397</v>
+        <v>0.4390426458084115</v>
       </c>
       <c r="BK9" t="n">
-        <v>65.66704467283006</v>
+        <v>0.01967862200541612</v>
       </c>
       <c r="BL9" t="n">
-        <v>12.77005612633976</v>
+        <v>0.01907703281096426</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>64.90469963240626</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>24.42358198018362</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>7518.27914252001</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>5.487645818432918e-05</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>0.7448686685247691</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>6.130733542514624</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>2.765584042406658</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>2108.021327332591</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>8301.704358866094</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>0.446983401187392</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>31.5071680029066</v>
       </c>
     </row>
     <row r="10">
@@ -2423,67 +2764,67 @@
         <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>94750.91620065976</v>
+        <v>86063.73265902369</v>
       </c>
       <c r="C10" t="n">
-        <v>0.2147286655549062</v>
+        <v>0.191005800350325</v>
       </c>
       <c r="D10" t="n">
         <v>0.3602129724167135</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2082643961585085</v>
+        <v>0.2048970581857102</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1980314361636714</v>
+        <v>0.20688468746942</v>
       </c>
       <c r="G10" t="n">
-        <v>0.05683291464323689</v>
+        <v>0.0493172562464534</v>
       </c>
       <c r="H10" t="n">
-        <v>328.5997687297807</v>
+        <v>320.7264701077852</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1539471839894275</v>
+        <v>0.2189471839894276</v>
       </c>
       <c r="J10" t="n">
-        <v>0.09052584854183726</v>
+        <v>0.1185258485418373</v>
       </c>
       <c r="K10" t="n">
-        <v>0.09329503520885959</v>
+        <v>0.0872920818671824</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1453986922775232</v>
+        <v>0.1629147417384677</v>
       </c>
       <c r="M10" t="n">
-        <v>0.8013868585829963</v>
+        <v>0.9415152542705523</v>
       </c>
       <c r="N10" t="n">
-        <v>0.3571708464703898</v>
+        <v>0.3408211523080106</v>
       </c>
       <c r="O10" t="n">
-        <v>0.09813784942267889</v>
+        <v>0.1021031810912819</v>
       </c>
       <c r="P10" t="n">
-        <v>1.32637472895426</v>
+        <v>1.422449343274217</v>
       </c>
       <c r="Q10" t="n">
-        <v>1.016383739454707</v>
+        <v>0.9433471210963443</v>
       </c>
       <c r="R10" t="n">
         <v>1.050337496602176</v>
       </c>
       <c r="S10" t="n">
-        <v>1.858313297084734</v>
+        <v>1.772525100340563</v>
       </c>
       <c r="T10" t="n">
-        <v>0.1551349112043872</v>
+        <v>0.1481834765970744</v>
       </c>
       <c r="U10" t="n">
-        <v>3.73429938093344</v>
+        <v>2.956111119543106</v>
       </c>
       <c r="V10" t="n">
-        <v>0.001247843023142831</v>
+        <v>0.001058819760157621</v>
       </c>
       <c r="W10" t="n">
         <v>0.002124738818796891</v>
@@ -2492,124 +2833,157 @@
         <v>-0.05254834829148167</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.2207722936743352</v>
+        <v>0.1975913831243319</v>
       </c>
       <c r="Z10" t="n">
-        <v>0.01636044038024676</v>
+        <v>0.02002278605174138</v>
       </c>
       <c r="AA10" t="n">
         <v>0.1009633328647785</v>
       </c>
       <c r="AB10" t="n">
-        <v>0.9267155457452458</v>
+        <v>0.8365695530895042</v>
       </c>
       <c r="AC10" t="n">
         <v>0.9365343331016135</v>
       </c>
       <c r="AD10" t="n">
-        <v>0.8659580612816291</v>
+        <v>0.8290025241710903</v>
       </c>
       <c r="AE10" t="n">
-        <v>0.8923096410177789</v>
+        <v>0.9024703487440867</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.7674540368462753</v>
+        <v>0.8088252917706893</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.8109950450585433</v>
+        <v>0.7949950450585432</v>
       </c>
       <c r="AH10" t="n">
-        <v>0.9223790496022315</v>
+        <v>0.7863790496022315</v>
       </c>
       <c r="AI10" t="n">
-        <v>0.1116959246208749</v>
+        <v>0.129742496478643</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0.3204904871161887</v>
+        <v>0.2950375334764932</v>
       </c>
       <c r="AK10" t="n">
         <v>0.3006763366605896</v>
       </c>
       <c r="AL10" t="n">
-        <v>1.61494525845166</v>
+        <v>1.21174525845166</v>
       </c>
       <c r="AM10" t="n">
-        <v>26.8500477813434</v>
+        <v>0.3679326704440395</v>
       </c>
       <c r="AN10" t="n">
-        <v>0.5783730569773728</v>
+        <v>0.5970275810763466</v>
       </c>
       <c r="AO10" t="n">
-        <v>0.1963347677556326</v>
+        <v>95.31870926307622</v>
       </c>
       <c r="AP10" t="n">
-        <v>3.096976873919347</v>
+        <v>13.69303984928001</v>
       </c>
       <c r="AQ10" t="n">
-        <v>1646.802575592755</v>
+        <v>36.43714450036873</v>
       </c>
       <c r="AR10" t="n">
-        <v>7892.400301387221</v>
+        <v>0.5350728741543768</v>
       </c>
       <c r="AS10" t="n">
-        <v>0.5011678835719341</v>
+        <v>0.1953232928337417</v>
       </c>
       <c r="AT10" t="n">
-        <v>0.3427989869238686</v>
+        <v>3.094805787868973</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.5618318773716742</v>
+        <v>1719.399279887451</v>
       </c>
       <c r="AV10" t="n">
-        <v>9.251727851443732</v>
+        <v>9317.195616169938</v>
       </c>
       <c r="AW10" t="n">
-        <v>1.067085810631782</v>
+        <v>0.5282603022929616</v>
       </c>
       <c r="AX10" t="n">
-        <v>1.42940116611299</v>
+        <v>11.45572852479816</v>
       </c>
       <c r="AY10" t="n">
-        <v>1.042410382318659</v>
+        <v>0.9549227668956469</v>
       </c>
       <c r="AZ10" t="n">
-        <v>49.5466480560044</v>
+        <v>1.284252837222767</v>
       </c>
       <c r="BA10" t="n">
-        <v>0.2599357836423797</v>
+        <v>0.9507327288977089</v>
       </c>
       <c r="BB10" t="n">
-        <v>0.1729933726003475</v>
+        <v>50.94742287932382</v>
       </c>
       <c r="BC10" t="n">
-        <v>0.9690841629903162</v>
+        <v>0.211970504150144</v>
       </c>
       <c r="BD10" t="n">
-        <v>10.07444894670207</v>
+        <v>0.162780624786241</v>
       </c>
       <c r="BE10" t="n">
-        <v>4.418093155567163</v>
+        <v>1.008422472299964</v>
       </c>
       <c r="BF10" t="n">
-        <v>0.600978319610599</v>
+        <v>10.24453888168103</v>
       </c>
       <c r="BG10" t="n">
-        <v>0.09993286987915735</v>
+        <v>4.123812267985933</v>
       </c>
       <c r="BH10" t="n">
-        <v>0.4696024040831009</v>
+        <v>0.2667973279374896</v>
       </c>
       <c r="BI10" t="n">
-        <v>0.03346770214080722</v>
+        <v>0.09176511292961134</v>
       </c>
       <c r="BJ10" t="n">
-        <v>0.01733218295721742</v>
+        <v>0.4715530502753136</v>
       </c>
       <c r="BK10" t="n">
-        <v>76.80448180695319</v>
+        <v>0.02938746124328392</v>
       </c>
       <c r="BL10" t="n">
-        <v>13.09701493002105</v>
+        <v>0.02193472714350862</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>59.41699221199007</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>30.40708894830952</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>8155.369731084467</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>5.627819307210342e-05</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>0.73734704826693</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>6.752078031201466</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>2.769742812012395</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>2167.017332329799</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>9298.465944655261</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>0.5268123156801273</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>26.80859991595297</v>
       </c>
     </row>
     <row r="11">
@@ -2617,193 +2991,226 @@
         <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>86794.90164921099</v>
+        <v>92046.1637342161</v>
       </c>
       <c r="C11" t="n">
-        <v>0.2086511647651165</v>
+        <v>0.1772409550030191</v>
       </c>
       <c r="D11" t="n">
-        <v>0.3643369130030688</v>
+        <v>0.3579533748586489</v>
       </c>
       <c r="E11" t="n">
-        <v>0.2137135996987267</v>
+        <v>0.2068041286701686</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2001536889947531</v>
+        <v>0.2118015174048373</v>
       </c>
       <c r="G11" t="n">
-        <v>0.04351865807369707</v>
+        <v>0.0453237931626411</v>
       </c>
       <c r="H11" t="n">
-        <v>312.1820742683216</v>
+        <v>348.6785258820481</v>
       </c>
       <c r="I11" t="n">
-        <v>0.2353970988628201</v>
+        <v>0.1573970988628201</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1050617050602146</v>
+        <v>0.0970617050602146</v>
       </c>
       <c r="K11" t="n">
-        <v>0.08650596566771454</v>
+        <v>0.09262549990944817</v>
       </c>
       <c r="L11" t="n">
-        <v>0.1205433410447259</v>
+        <v>0.1672528062739112</v>
       </c>
       <c r="M11" t="n">
-        <v>0.9262668767805794</v>
+        <v>1.031363173546247</v>
       </c>
       <c r="N11" t="n">
-        <v>0.4888256443866488</v>
+        <v>0.4724759502242697</v>
       </c>
       <c r="O11" t="n">
-        <v>0.1006577674676216</v>
+        <v>0.08876177246181263</v>
       </c>
       <c r="P11" t="n">
-        <v>1.258286263189961</v>
+        <v>1.210248956029982</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.7469078187115017</v>
+        <v>0.9660176737865892</v>
       </c>
       <c r="R11" t="n">
-        <v>1.068300275532508</v>
+        <v>0.8843129510188895</v>
       </c>
       <c r="S11" t="n">
-        <v>2.256472024029684</v>
+        <v>2.084895630541342</v>
       </c>
       <c r="T11" t="n">
-        <v>0.1304470503875068</v>
+        <v>0.1158931827772177</v>
       </c>
       <c r="U11" t="n">
-        <v>3.626337470232873</v>
+        <v>3.475606213151645</v>
       </c>
       <c r="V11" t="n">
-        <v>0.001064686279366211</v>
+        <v>0.001005501162828068</v>
       </c>
       <c r="W11" t="n">
-        <v>0.00199361799156342</v>
+        <v>0.002627951086779965</v>
       </c>
       <c r="X11" t="n">
-        <v>-0.05057875615400295</v>
+        <v>-0.05375002647638144</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.2083057980634986</v>
+        <v>0.1909936475651779</v>
       </c>
       <c r="Z11" t="n">
-        <v>0.02642743476417509</v>
+        <v>0.01934006304238763</v>
       </c>
       <c r="AA11" t="n">
-        <v>0.09408732610751554</v>
+        <v>0.09983393282004602</v>
       </c>
       <c r="AB11" t="n">
-        <v>0.8714269724823661</v>
+        <v>0.8938211029238522</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.9455643072007834</v>
+        <v>0.9180584077561497</v>
       </c>
       <c r="AD11" t="n">
-        <v>0.8767563998110182</v>
+        <v>0.8548307078897042</v>
       </c>
       <c r="AE11" t="n">
-        <v>0.9184514697512154</v>
+        <v>0.860097745778136</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.8186307093918104</v>
+        <v>0.7539959487908318</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.7546305184439824</v>
+        <v>0.8666305184439824</v>
       </c>
       <c r="AH11" t="n">
-        <v>0.862389592548926</v>
+        <v>0.913389592548926</v>
       </c>
       <c r="AI11" t="n">
-        <v>0.1129996669940811</v>
+        <v>0.1105505258660062</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0.2886034267103514</v>
+        <v>0.3014429877235558</v>
       </c>
       <c r="AK11" t="n">
-        <v>0.3510650663811189</v>
+        <v>0.3430721857451025</v>
       </c>
       <c r="AL11" t="n">
-        <v>1.160927765339252</v>
+        <v>1.621727765339252</v>
       </c>
       <c r="AM11" t="n">
-        <v>30.47051711636138</v>
+        <v>0.3505794817606436</v>
       </c>
       <c r="AN11" t="n">
-        <v>0.5436098686118952</v>
+        <v>0.5444497575345824</v>
       </c>
       <c r="AO11" t="n">
-        <v>0.2382270753753387</v>
+        <v>80.80360589345364</v>
       </c>
       <c r="AP11" t="n">
-        <v>3.013848054990484</v>
+        <v>12.4959360507932</v>
       </c>
       <c r="AQ11" t="n">
-        <v>1584.118598666035</v>
+        <v>29.97610269679806</v>
       </c>
       <c r="AR11" t="n">
-        <v>7719.515671921023</v>
+        <v>0.6128198534372533</v>
       </c>
       <c r="AS11" t="n">
-        <v>0.491946019204109</v>
+        <v>0.1888062016460452</v>
       </c>
       <c r="AT11" t="n">
-        <v>0.3614269094677607</v>
+        <v>2.646832516373479</v>
       </c>
       <c r="AU11" t="n">
-        <v>0.5006420134934636</v>
+        <v>1532.137196467065</v>
       </c>
       <c r="AV11" t="n">
-        <v>10.12812289156891</v>
+        <v>8632.445596346202</v>
       </c>
       <c r="AW11" t="n">
-        <v>0.9971614195791279</v>
+        <v>0.5149661759306247</v>
       </c>
       <c r="AX11" t="n">
-        <v>1.157093022031957</v>
+        <v>9.596251466861393</v>
       </c>
       <c r="AY11" t="n">
-        <v>1.193760953824286</v>
+        <v>1.148284346059551</v>
       </c>
       <c r="AZ11" t="n">
-        <v>52.16248607274127</v>
+        <v>1.385681591075611</v>
       </c>
       <c r="BA11" t="n">
-        <v>0.2331381393321275</v>
+        <v>1.151242464776354</v>
       </c>
       <c r="BB11" t="n">
-        <v>0.1802638158332852</v>
+        <v>52.10370318781098</v>
       </c>
       <c r="BC11" t="n">
-        <v>1.00659414692309</v>
+        <v>0.2488581087073575</v>
       </c>
       <c r="BD11" t="n">
-        <v>11.87003668628784</v>
+        <v>0.1403778785682522</v>
       </c>
       <c r="BE11" t="n">
-        <v>4.002026863680451</v>
+        <v>1.002061608126269</v>
       </c>
       <c r="BF11" t="n">
-        <v>0.4180282082047564</v>
+        <v>11.52334485233012</v>
       </c>
       <c r="BG11" t="n">
-        <v>0.08648907651223357</v>
+        <v>3.257201510761065</v>
       </c>
       <c r="BH11" t="n">
-        <v>0.4399802544741194</v>
+        <v>0.1826568078876027</v>
       </c>
       <c r="BI11" t="n">
-        <v>0.02039635586404064</v>
+        <v>0.1037791653579657</v>
       </c>
       <c r="BJ11" t="n">
-        <v>0.01966754181947924</v>
+        <v>0.4049625428124938</v>
       </c>
       <c r="BK11" t="n">
-        <v>73.60619551643937</v>
+        <v>0.007562690187870581</v>
       </c>
       <c r="BL11" t="n">
-        <v>11.3519858781555</v>
+        <v>0.01692252220193575</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>51.89604658767207</v>
+      </c>
+      <c r="BN11" t="n">
+        <v>28.73380964507528</v>
+      </c>
+      <c r="BO11" t="n">
+        <v>7801.96681366235</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>4.862423141450689e-05</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>0.7524313094945082</v>
+      </c>
+      <c r="BR11" t="n">
+        <v>7.656848065634634</v>
+      </c>
+      <c r="BS11" t="n">
+        <v>3.223785346948572</v>
+      </c>
+      <c r="BT11" t="n">
+        <v>1923.313458433587</v>
+      </c>
+      <c r="BU11" t="n">
+        <v>7956.427826071604</v>
+      </c>
+      <c r="BV11" t="n">
+        <v>0.4947145110138218</v>
+      </c>
+      <c r="BW11" t="n">
+        <v>34.91111350730139</v>
       </c>
     </row>
     <row r="12">
@@ -2811,193 +3218,226 @@
         <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>79758.46455672588</v>
+        <v>81731.55058755084</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1841866794561577</v>
+        <v>0.2034622861020961</v>
       </c>
       <c r="D12" t="n">
-        <v>0.3711114552337078</v>
+        <v>0.3672510026236806</v>
       </c>
       <c r="E12" t="n">
-        <v>0.2040567813706302</v>
+        <v>0.2122339701268834</v>
       </c>
       <c r="F12" t="n">
-        <v>0.1973730107277107</v>
+        <v>0.2042972539967521</v>
       </c>
       <c r="G12" t="n">
-        <v>0.04120176185892341</v>
+        <v>0.03469620740163024</v>
       </c>
       <c r="H12" t="n">
         <v>346.8198374390021</v>
       </c>
       <c r="I12" t="n">
-        <v>0.2508178659326675</v>
+        <v>0.2118178659326675</v>
       </c>
       <c r="J12" t="n">
         <v>0.08009519302152898</v>
       </c>
       <c r="K12" t="n">
-        <v>0.09157478330675467</v>
+        <v>0.09581275908580149</v>
       </c>
       <c r="L12" t="n">
-        <v>0.1640142262018686</v>
+        <v>0.140659493587276</v>
       </c>
       <c r="M12" t="n">
-        <v>0.8131842684422065</v>
+        <v>0.7431200705984284</v>
       </c>
       <c r="N12" t="n">
-        <v>0.337234507262651</v>
+        <v>0.3862835897497883</v>
       </c>
       <c r="O12" t="n">
-        <v>0.1167143252954797</v>
+        <v>0.08499167194665581</v>
       </c>
       <c r="P12" t="n">
-        <v>1.241672258848524</v>
+        <v>1.049523030208608</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.9584412168443029</v>
+        <v>0.8488862893067592</v>
       </c>
       <c r="R12" t="n">
-        <v>0.8595660547156367</v>
+        <v>0.7859711249101893</v>
       </c>
       <c r="S12" t="n">
-        <v>2.521428145379891</v>
+        <v>2.178275358403208</v>
       </c>
       <c r="T12" t="n">
-        <v>0.1324810825524857</v>
+        <v>0.1353152380051858</v>
       </c>
       <c r="U12" t="n">
-        <v>4.020058696876928</v>
+        <v>3.221704153340419</v>
       </c>
       <c r="V12" t="n">
-        <v>0.0009271519492096192</v>
+        <v>0.001076365508794658</v>
       </c>
       <c r="W12" t="n">
-        <v>0.002165877422309804</v>
+        <v>0.002315515774587243</v>
       </c>
       <c r="X12" t="n">
-        <v>-0.06084201013954599</v>
+        <v>-0.05751854233179692</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.1840957089791968</v>
+        <v>0.2355246362280073</v>
       </c>
       <c r="Z12" t="n">
-        <v>0.02432152182430029</v>
+        <v>0.02150028739357042</v>
       </c>
       <c r="AA12" t="n">
-        <v>0.09915880777873645</v>
+        <v>0.09799273169372294</v>
       </c>
       <c r="AB12" t="n">
-        <v>0.7965989262304435</v>
+        <v>0.8804663172080454</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.9502038447947875</v>
+        <v>0.9541290277264163</v>
       </c>
       <c r="AD12" t="n">
-        <v>0.8496691100031784</v>
+        <v>0.860846717743053</v>
       </c>
       <c r="AE12" t="n">
-        <v>0.8244765178892479</v>
+        <v>0.915193911379294</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.7928013600954433</v>
+        <v>0.7864959782170557</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.7421980184645999</v>
+        <v>0.7581980184645999</v>
       </c>
       <c r="AH12" t="n">
-        <v>0.7843534905491777</v>
+        <v>0.8013534905491777</v>
       </c>
       <c r="AI12" t="n">
-        <v>0.1053295126685243</v>
+        <v>0.1152387286364352</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0.2576730367512008</v>
+        <v>0.3216598290527042</v>
       </c>
       <c r="AK12" t="n">
-        <v>0.3614523169303648</v>
+        <v>0.4144413067495473</v>
       </c>
       <c r="AL12" t="n">
-        <v>1.460985767791799</v>
+        <v>1.691385767791799</v>
       </c>
       <c r="AM12" t="n">
-        <v>28.14316240701475</v>
+        <v>0.326834288461184</v>
       </c>
       <c r="AN12" t="n">
-        <v>0.5989394473736844</v>
+        <v>0.6210387062178073</v>
       </c>
       <c r="AO12" t="n">
-        <v>0.2181716275729057</v>
+        <v>86.96837137048541</v>
       </c>
       <c r="AP12" t="n">
-        <v>2.772154962078119</v>
+        <v>12.02087895164443</v>
       </c>
       <c r="AQ12" t="n">
-        <v>1973.009898728521</v>
+        <v>26.01744873156638</v>
       </c>
       <c r="AR12" t="n">
-        <v>8062.595709680583</v>
+        <v>0.5571834580030812</v>
       </c>
       <c r="AS12" t="n">
-        <v>0.4798850013003684</v>
+        <v>0.2064514838405339</v>
       </c>
       <c r="AT12" t="n">
-        <v>0.3572412359874582</v>
+        <v>3.373780314539769</v>
       </c>
       <c r="AU12" t="n">
-        <v>0.6247314764623599</v>
+        <v>1980.449541934865</v>
       </c>
       <c r="AV12" t="n">
-        <v>10.3916285516887</v>
+        <v>8192.759950151374</v>
       </c>
       <c r="AW12" t="n">
-        <v>1.089413416819823</v>
+        <v>0.4481368625848038</v>
       </c>
       <c r="AX12" t="n">
-        <v>1.279727853330424</v>
+        <v>10.74362533741349</v>
       </c>
       <c r="AY12" t="n">
-        <v>0.9873839690450084</v>
+        <v>1.019575849313745</v>
       </c>
       <c r="AZ12" t="n">
-        <v>50.08331857476363</v>
+        <v>1.483860353236059</v>
       </c>
       <c r="BA12" t="n">
-        <v>0.2452827799516978</v>
+        <v>0.9963180294390573</v>
       </c>
       <c r="BB12" t="n">
-        <v>0.2010739728992679</v>
+        <v>51.51398086684955</v>
       </c>
       <c r="BC12" t="n">
-        <v>1.060349691849894</v>
+        <v>0.2204645286661866</v>
       </c>
       <c r="BD12" t="n">
-        <v>12.68489743124014</v>
+        <v>0.1749641372575125</v>
       </c>
       <c r="BE12" t="n">
-        <v>3.440010153564556</v>
+        <v>1.040169351967284</v>
       </c>
       <c r="BF12" t="n">
-        <v>0.7161667141433128</v>
+        <v>9.821382667026855</v>
       </c>
       <c r="BG12" t="n">
-        <v>0.09004607713580814</v>
+        <v>4.173958061670303</v>
       </c>
       <c r="BH12" t="n">
-        <v>0.4335421663096016</v>
+        <v>0.5385445299497382</v>
       </c>
       <c r="BI12" t="n">
-        <v>0.005889272034392752</v>
+        <v>0.09836753503180477</v>
       </c>
       <c r="BJ12" t="n">
-        <v>0.01816066329267608</v>
+        <v>0.3981240787910647</v>
       </c>
       <c r="BK12" t="n">
-        <v>82.99718517606135</v>
+        <v>0.02493915885414301</v>
       </c>
       <c r="BL12" t="n">
-        <v>14.09976500914031</v>
+        <v>0.02030292189953204</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>60.45378425863147</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>29.98597147086961</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>7898.849465169814</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>6.318594965714537e-05</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>0.7278491335295697</v>
+      </c>
+      <c r="BR12" t="n">
+        <v>6.488284494732047</v>
+      </c>
+      <c r="BS12" t="n">
+        <v>2.910215724095681</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>1768.952519151304</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>8614.235686358717</v>
+      </c>
+      <c r="BV12" t="n">
+        <v>0.583571542991115</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>31.15033230735995</v>
       </c>
     </row>
   </sheetData>

</xml_diff>